<commit_message>
Reduce product image downloads with WebP and background loading
</commit_message>
<xml_diff>
--- a/games/reaction-speed-test/config/game_config.xlsx
+++ b/games/reaction-speed-test/config/game_config.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameSettings" sheetId="1" r:id="R8f350d4b771241c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="2" r:id="Rba8157522e1640f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="Rfa0c4dee75a948d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stimuli" sheetId="4" r:id="R33106b637c884fbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InfiniteMode" sheetId="5" r:id="Rc4a02161b2284cae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rf7266b144e664ae9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="7" r:id="Rfd8c638c336440f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="8" r:id="R7ba852def13d40a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Text" sheetId="9" r:id="R802f8cdad4b54acf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameSettings" sheetId="1" r:id="R1018833403f44e95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="2" r:id="R93903e62e0934794"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="Rabd1820944804776"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stimuli" sheetId="4" r:id="R6242bc31995746af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InfiniteMode" sheetId="5" r:id="Rd2fc64fd20674a48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R674af38947484328"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="7" r:id="Rab5973a7a46147da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="8" r:id="R3155b86c4c124395"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Text" sheetId="9" r:id="Rf503062fbd674bda"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10023,7 +10023,7 @@
         <x:v>target</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>ABT+2.png</x:v>
+        <x:v>ABT+2.webp</x:v>
       </x:c>
       <x:c r="D2" t="b">
         <x:v>1</x:v>
@@ -10040,7 +10040,7 @@
         <x:v>target</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>BBB+1.png</x:v>
+        <x:v>BBB+1.webp</x:v>
       </x:c>
       <x:c r="D3" t="b">
         <x:v>1</x:v>
@@ -10057,7 +10057,7 @@
         <x:v>target</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>MTT+10.png</x:v>
+        <x:v>MTT+10.webp</x:v>
       </x:c>
       <x:c r="D4" t="b">
         <x:v>1</x:v>
@@ -10074,7 +10074,7 @@
         <x:v>target</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>NAP+1.png</x:v>
+        <x:v>NAP+1.webp</x:v>
       </x:c>
       <x:c r="D5" t="b">
         <x:v>1</x:v>
@@ -10091,7 +10091,7 @@
         <x:v>target</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>PPA+1.png</x:v>
+        <x:v>PPA+1.webp</x:v>
       </x:c>
       <x:c r="D6" t="b">
         <x:v>1</x:v>
@@ -10125,7 +10125,7 @@
         <x:v>target</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>BBB+1.png</x:v>
+        <x:v>BBB+1.webp</x:v>
       </x:c>
       <x:c r="D8" t="b">
         <x:v>1</x:v>
@@ -10142,7 +10142,7 @@
         <x:v>target</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>MTT+10.png</x:v>
+        <x:v>MTT+10.webp</x:v>
       </x:c>
       <x:c r="D9" t="b">
         <x:v>1</x:v>
@@ -10159,7 +10159,7 @@
         <x:v>target</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>NAP+1.png</x:v>
+        <x:v>NAP+1.webp</x:v>
       </x:c>
       <x:c r="D10" t="b">
         <x:v>1</x:v>
@@ -10176,7 +10176,7 @@
         <x:v>target</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>PPA+1.png</x:v>
+        <x:v>PPA+1.webp</x:v>
       </x:c>
       <x:c r="D11" t="b">
         <x:v>1</x:v>
@@ -10193,7 +10193,7 @@
         <x:v>target</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>QSS+8.png</x:v>
+        <x:v>QSS+8.webp</x:v>
       </x:c>
       <x:c r="D12" s="1" t="b">
         <x:v>1</x:v>
@@ -10210,7 +10210,7 @@
         <x:v>target</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>SDD+10.png</x:v>
+        <x:v>SDD+10.webp</x:v>
       </x:c>
       <x:c r="D13" s="1" t="b">
         <x:v>1</x:v>
@@ -10227,7 +10227,7 @@
         <x:v>target</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>YSS+2.png</x:v>
+        <x:v>YSS+2.webp</x:v>
       </x:c>
       <x:c r="D14" s="1" t="b">
         <x:v>1</x:v>

</xml_diff>

<commit_message>
Improve single-screen game layouts and replace star cue with background jellyfish
</commit_message>
<xml_diff>
--- a/games/reaction-speed-test/config/game_config.xlsx
+++ b/games/reaction-speed-test/config/game_config.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameSettings" sheetId="1" r:id="R1018833403f44e95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="2" r:id="R93903e62e0934794"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="Rabd1820944804776"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stimuli" sheetId="4" r:id="R6242bc31995746af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InfiniteMode" sheetId="5" r:id="Rd2fc64fd20674a48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="R674af38947484328"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="7" r:id="Rab5973a7a46147da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="8" r:id="R3155b86c4c124395"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Text" sheetId="9" r:id="Rf503062fbd674bda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameSettings" sheetId="1" r:id="R72f4aad1411042e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="2" r:id="R2514fc28e82a44ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R47b0226a1c304036"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stimuli" sheetId="4" r:id="R3eed6c1e6ac34829"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InfiniteMode" sheetId="5" r:id="R9b5359be32b34b39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rdda6b7ef4a4e47a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="7" r:id="Rbad9383c31034f9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="8" r:id="R0eefa96c359f4410"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Text" sheetId="9" r:id="Rccc079b5353b42c2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3262,7 +3262,7 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B42" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C42" t="str">
         <x:v>catalogue-41</x:v>
@@ -3330,7 +3330,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="B43" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C43" t="str">
         <x:v>catalogue-42</x:v>
@@ -3398,7 +3398,7 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B44" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C44" t="str">
         <x:v>catalogue-44</x:v>
@@ -3466,7 +3466,7 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B45" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C45" t="str">
         <x:v>catalogue-45</x:v>
@@ -3534,7 +3534,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="B46" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C46" t="str">
         <x:v>catalogue-49</x:v>
@@ -3602,7 +3602,7 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="B47" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C47" t="str">
         <x:v>catalogue-50</x:v>
@@ -3670,7 +3670,7 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="B48" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C48" t="str">
         <x:v>catalogue-55</x:v>
@@ -3738,7 +3738,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B49" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C49" t="str">
         <x:v>catalogue-56</x:v>
@@ -3806,7 +3806,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B50" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C50" t="str">
         <x:v>catalogue-57</x:v>
@@ -3874,7 +3874,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="B51" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C51" t="str">
         <x:v>catalogue-78</x:v>
@@ -3942,7 +3942,7 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="B52" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C52" t="str">
         <x:v>catalogue-52</x:v>
@@ -4010,7 +4010,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="B53" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C53" t="str">
         <x:v>catalogue-53</x:v>
@@ -4078,7 +4078,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="B54" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C54" t="str">
         <x:v>catalogue-60</x:v>
@@ -4146,7 +4146,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="B55" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C55" t="str">
         <x:v>catalogue-61</x:v>
@@ -4214,7 +4214,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C56" t="str">
         <x:v>catalogue-64</x:v>
@@ -4282,7 +4282,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C57" t="str">
         <x:v>catalogue-65</x:v>
@@ -4350,7 +4350,7 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C58" t="str">
         <x:v>catalogue-66</x:v>
@@ -4418,7 +4418,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C59" t="str">
         <x:v>catalogue-43</x:v>
@@ -4486,7 +4486,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C60" t="str">
         <x:v>catalogue-51</x:v>
@@ -4554,7 +4554,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C61" t="str">
         <x:v>catalogue-54</x:v>
@@ -4622,7 +4622,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C62" t="str">
         <x:v>catalogue-76</x:v>
@@ -4690,7 +4690,7 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C63" t="str">
         <x:v>catalogue-77</x:v>
@@ -4758,7 +4758,7 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C64" t="str">
         <x:v>catalogue-48</x:v>
@@ -4826,7 +4826,7 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C65" t="str">
         <x:v>catalogue-62</x:v>
@@ -4894,7 +4894,7 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C66" t="str">
         <x:v>catalogue-63</x:v>
@@ -4962,7 +4962,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>排除色環／單一商品／星星有</x:v>
+        <x:v>排除色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C67" t="str">
         <x:v>catalogue-74</x:v>
@@ -5030,7 +5030,7 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>單一色環／排除商品／星星有</x:v>
+        <x:v>單一色環／排除商品／水母有</x:v>
       </x:c>
       <x:c r="C68" t="str">
         <x:v>catalogue-75</x:v>
@@ -5098,7 +5098,7 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>排除色環／單一商品／星星無</x:v>
+        <x:v>排除色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C69" t="str">
         <x:v>catalogue-100</x:v>
@@ -5166,7 +5166,7 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C70" t="str">
         <x:v>catalogue-46</x:v>
@@ -5234,7 +5234,7 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C71" t="str">
         <x:v>catalogue-47</x:v>
@@ -5302,7 +5302,7 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>多種色環／單一商品／星星無</x:v>
+        <x:v>多種色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C72" t="str">
         <x:v>catalogue-58</x:v>
@@ -5370,7 +5370,7 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>單一色環／多種商品／星星無</x:v>
+        <x:v>單一色環／多種商品／水母無</x:v>
       </x:c>
       <x:c r="C73" t="str">
         <x:v>catalogue-59</x:v>
@@ -5438,7 +5438,7 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C74" t="str">
         <x:v>catalogue-68</x:v>
@@ -5506,7 +5506,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C75" t="str">
         <x:v>catalogue-69</x:v>
@@ -5574,7 +5574,7 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C76" t="str">
         <x:v>catalogue-71</x:v>
@@ -5642,7 +5642,7 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C77" t="str">
         <x:v>catalogue-72</x:v>
@@ -5710,7 +5710,7 @@
         <x:v>77</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C78" t="str">
         <x:v>catalogue-80</x:v>
@@ -5778,7 +5778,7 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C79" t="str">
         <x:v>catalogue-81</x:v>
@@ -5846,7 +5846,7 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C80" t="str">
         <x:v>catalogue-86</x:v>
@@ -5914,7 +5914,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C81" t="str">
         <x:v>catalogue-87</x:v>
@@ -5982,7 +5982,7 @@
         <x:v>81</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C82" t="str">
         <x:v>catalogue-88</x:v>
@@ -6050,7 +6050,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C83" t="str">
         <x:v>catalogue-90</x:v>
@@ -6118,7 +6118,7 @@
         <x:v>83</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C84" t="str">
         <x:v>catalogue-91</x:v>
@@ -6186,7 +6186,7 @@
         <x:v>84</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C85" t="str">
         <x:v>catalogue-96</x:v>
@@ -6254,7 +6254,7 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C86" t="str">
         <x:v>catalogue-97</x:v>
@@ -6322,7 +6322,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C87" t="str">
         <x:v>catalogue-98</x:v>
@@ -6390,7 +6390,7 @@
         <x:v>87</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>多種色環／單一商品／星星無</x:v>
+        <x:v>多種色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C88" t="str">
         <x:v>catalogue-83</x:v>
@@ -6458,7 +6458,7 @@
         <x:v>88</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>多種色環／單一商品／星星無</x:v>
+        <x:v>多種色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C89" t="str">
         <x:v>catalogue-84</x:v>
@@ -6526,7 +6526,7 @@
         <x:v>89</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>單一色環／多種商品／星星無</x:v>
+        <x:v>單一色環／多種商品／水母無</x:v>
       </x:c>
       <x:c r="C90" t="str">
         <x:v>catalogue-93</x:v>
@@ -6594,7 +6594,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>單一色環／多種商品／星星無</x:v>
+        <x:v>單一色環／多種商品／水母無</x:v>
       </x:c>
       <x:c r="C91" t="str">
         <x:v>catalogue-94</x:v>
@@ -6662,7 +6662,7 @@
         <x:v>91</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C92" t="str">
         <x:v>catalogue-67</x:v>
@@ -6730,7 +6730,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C93" t="str">
         <x:v>catalogue-70</x:v>
@@ -6798,7 +6798,7 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C94" t="str">
         <x:v>catalogue-82</x:v>
@@ -6866,7 +6866,7 @@
         <x:v>94</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C95" t="str">
         <x:v>catalogue-85</x:v>
@@ -6934,7 +6934,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C96" t="str">
         <x:v>catalogue-92</x:v>
@@ -7002,7 +7002,7 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C97" t="str">
         <x:v>catalogue-95</x:v>
@@ -7070,7 +7070,7 @@
         <x:v>97</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>多種色環／單一商品／星星無</x:v>
+        <x:v>多種色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C98" t="str">
         <x:v>catalogue-79</x:v>
@@ -7138,7 +7138,7 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>單一色環／多種商品／星星無</x:v>
+        <x:v>單一色環／多種商品／水母無</x:v>
       </x:c>
       <x:c r="C99" t="str">
         <x:v>catalogue-89</x:v>
@@ -7206,7 +7206,7 @@
         <x:v>99</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>多種色環／多種商品／星星有</x:v>
+        <x:v>多種色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C100" t="str">
         <x:v>catalogue-73</x:v>
@@ -7274,7 +7274,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>多種色環／多種商品／星星無</x:v>
+        <x:v>多種色環／多種商品／水母無</x:v>
       </x:c>
       <x:c r="C101" t="str">
         <x:v>catalogue-99</x:v>
@@ -7445,7 +7445,7 @@
         <x:v>星星禁點</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>有灰色星星時，甚麼都別點。沒有星星時，只點金色商品。</x:v>
+        <x:v>有背景水母時，甚麼都別點。沒有星星時，只點金色商品。</x:v>
       </x:c>
       <x:c r="D7" t="str">
         <x:v>{"targetType":"gold","distractorCondition":"absent"}</x:v>
@@ -7507,7 +7507,7 @@
         <x:v>綜合模式</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>前半：左側金色或右側棕色；後半：有灰色星星時甚麼都別點，沒有時只點金色商品。</x:v>
+        <x:v>前半：左側金色或右側棕色；後半：有背景水母時甚麼都別點，沒有時只點金色商品。</x:v>
       </x:c>
       <x:c r="D11" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold","positionCondition":"left"},{"targetType":"brown","positionCondition":"right"}]}}</x:v>
@@ -7524,7 +7524,7 @@
         <x:v>無干擾時點擊</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>只有沒有灰色星星時，才點擊金色商品。</x:v>
+        <x:v>只有沒有背景水母時，才點擊金色商品。</x:v>
       </x:c>
       <x:c r="D12" t="str">
         <x:v>{"targetType":"gold","distractorCondition":"absent"}</x:v>
@@ -8136,10 +8136,10 @@
         <x:v>catalogue-41</x:v>
       </x:c>
       <x:c r="B53" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C53" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 或 （畫面有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 或 （背景出現水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D53" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"compoundCondition":{"op":"any","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}]}}</x:v>
@@ -8151,10 +8151,10 @@
         <x:v>catalogue-42</x:v>
       </x:c>
       <x:c r="B54" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C54" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 或 （畫面沒有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 或 （背景沒有水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D54" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"compoundCondition":{"op":"any","conditions":[{"positionCondition":"left"},{"distractorCondition":"absent"}]}}]}}]}}</x:v>
@@ -8166,10 +8166,10 @@
         <x:v>catalogue-43</x:v>
       </x:c>
       <x:c r="B55" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C55" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （商品是 ABT+2）） 而且 （（出現在左半邊） 而且 （畫面有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （商品是 ABT+2）） 而且 （（出現在左半邊） 而且 （背景出現水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D55" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"targetShape":"circle"}]}},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}</x:v>
@@ -8181,10 +8181,10 @@
         <x:v>catalogue-44</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C56" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （出現在左半邊）） 或 （（商品是 ABT+2） 或 （畫面有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （出現在左半邊）） 或 （（商品是 ABT+2） 或 （背景出現水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D56" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"positionCondition":"left"}]}},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"distractorCondition":"present"}]}}]}}</x:v>
@@ -8196,10 +8196,10 @@
         <x:v>catalogue-45</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C57" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （畫面有灰色星星）） 或 （（商品是 ABT+2） 或 （出現在左半邊））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （背景出現水母）） 或 （（商品是 ABT+2） 或 （出現在左半邊））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D57" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"distractorCondition":"present"}]}},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"positionCondition":"left"}]}}]}}</x:v>
@@ -8211,10 +8211,10 @@
         <x:v>catalogue-46</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C58" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 或 （畫面有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 或 （背景出現水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D58" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"allowedTypes":["gold","brown"]},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"compoundCondition":{"op":"any","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}]}}</x:v>
@@ -8226,10 +8226,10 @@
         <x:v>catalogue-47</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C59" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （（出現在左半邊） 或 （畫面有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （（出現在左半邊） 或 （背景出現水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D59" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"compoundCondition":{"op":"any","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}]}}</x:v>
@@ -8241,10 +8241,10 @@
         <x:v>catalogue-48</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C60" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （商品是 ABT+2）） 而且 （（出現在左半邊） 而且 （畫面沒有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （商品是 ABT+2）） 而且 （（出現在左半邊） 而且 （背景沒有水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D60" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"targetShape":"circle"}]}},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"absent"}]}}]}}</x:v>
@@ -8256,10 +8256,10 @@
         <x:v>catalogue-49</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C61" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（商品是 ABT+2） 或 （出現在左半邊））） 而且 （畫面有灰色星星）。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（商品是 ABT+2） 或 （出現在左半邊））） 而且 （背景出現水母）。其餘不要點。</x:v>
       </x:c>
       <x:c r="D61" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"positionCondition":"left"}]}}]}},{"distractorCondition":"present"}]}}</x:v>
@@ -8271,10 +8271,10 @@
         <x:v>catalogue-50</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C62" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（商品是 ABT+2） 或 （畫面有灰色星星））） 而且 （出現在左半邊）。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（商品是 ABT+2） 或 （背景出現水母））） 而且 （出現在左半邊）。其餘不要點。</x:v>
       </x:c>
       <x:c r="D62" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"distractorCondition":"present"}]}}]}},{"positionCondition":"left"}]}}</x:v>
@@ -8286,10 +8286,10 @@
         <x:v>catalogue-51</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C63" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （（出現在左半邊） 而且 （畫面有灰色星星））） 或 （商品是 ABT+2）。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （（出現在左半邊） 而且 （背景出現水母））） 或 （商品是 ABT+2）。其餘不要點。</x:v>
       </x:c>
       <x:c r="D63" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}},{"targetShape":"circle"}]}}</x:v>
@@ -8301,10 +8301,10 @@
         <x:v>catalogue-52</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C64" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （出現在左半邊）） 或 （（商品是 ABT+2） 或 （畫面沒有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （出現在左半邊）） 或 （（商品是 ABT+2） 或 （背景沒有水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D64" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"positionCondition":"left"}]}},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"distractorCondition":"absent"}]}}]}}</x:v>
@@ -8316,10 +8316,10 @@
         <x:v>catalogue-53</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C65" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （畫面沒有灰色星星）） 或 （（商品是 ABT+2） 或 （出現在左半邊））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （背景沒有水母）） 或 （（商品是 ABT+2） 或 （出現在左半邊））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D65" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"distractorCondition":"absent"}]}},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"positionCondition":"left"}]}}]}}</x:v>
@@ -8331,10 +8331,10 @@
         <x:v>catalogue-54</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C66" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品是 ABT+2） 而且 （（出現在左半邊） 而且 （畫面有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品是 ABT+2） 而且 （（出現在左半邊） 而且 （背景出現水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D66" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"all","conditions":[{"targetShape":"circle"},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}]}}</x:v>
@@ -8346,10 +8346,10 @@
         <x:v>catalogue-55</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C67" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 而且 （出現在左半邊）） 或 （畫面有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 而且 （出現在左半邊）） 或 （背景出現水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D67" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetShape":"circle"},{"positionCondition":"left"}]}},{"distractorCondition":"present"}]}}]}}</x:v>
@@ -8361,10 +8361,10 @@
         <x:v>catalogue-56</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C68" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 而且 （畫面有灰色星星）） 或 （出現在左半邊））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 而且 （背景出現水母）） 或 （出現在左半邊））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D68" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetShape":"circle"},{"distractorCondition":"present"}]}},{"positionCondition":"left"}]}}]}}</x:v>
@@ -8376,10 +8376,10 @@
         <x:v>catalogue-57</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C69" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 而且 （畫面有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 而且 （背景出現水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D69" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}]}}</x:v>
@@ -8391,10 +8391,10 @@
         <x:v>catalogue-58</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>多種色環／單一商品／星星無</x:v>
+        <x:v>多種色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C70" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 或 （畫面沒有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 或 （背景沒有水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D70" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"allowedTypes":["gold","brown"]},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"compoundCondition":{"op":"any","conditions":[{"positionCondition":"left"},{"distractorCondition":"absent"}]}}]}}]}}</x:v>
@@ -8406,10 +8406,10 @@
         <x:v>catalogue-59</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>單一色環／多種商品／星星無</x:v>
+        <x:v>單一色環／多種商品／水母無</x:v>
       </x:c>
       <x:c r="C71" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （（出現在左半邊） 或 （畫面沒有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （（出現在左半邊） 或 （背景沒有水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D71" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"compoundCondition":{"op":"any","conditions":[{"positionCondition":"left"},{"distractorCondition":"absent"}]}}]}}]}}</x:v>
@@ -8421,10 +8421,10 @@
         <x:v>catalogue-60</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C72" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（商品是 ABT+2） 或 （出現在左半邊））） 而且 （畫面沒有灰色星星）。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（商品是 ABT+2） 或 （出現在左半邊））） 而且 （背景沒有水母）。其餘不要點。</x:v>
       </x:c>
       <x:c r="D72" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"positionCondition":"left"}]}}]}},{"distractorCondition":"absent"}]}}</x:v>
@@ -8436,10 +8436,10 @@
         <x:v>catalogue-61</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C73" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（商品是 ABT+2） 或 （畫面沒有灰色星星））） 而且 （出現在左半邊）。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（商品是 ABT+2） 或 （背景沒有水母））） 而且 （出現在左半邊）。其餘不要點。</x:v>
       </x:c>
       <x:c r="D73" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"distractorCondition":"absent"}]}}]}},{"positionCondition":"left"}]}}</x:v>
@@ -8451,10 +8451,10 @@
         <x:v>catalogue-62</x:v>
       </x:c>
       <x:c r="B74" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （（出現在左半邊） 而且 （畫面沒有灰色星星））） 或 （商品是 ABT+2）。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （（出現在左半邊） 而且 （背景沒有水母））） 或 （商品是 ABT+2）。其餘不要點。</x:v>
       </x:c>
       <x:c r="D74" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"absent"}]}}]}},{"targetShape":"circle"}]}}</x:v>
@@ -8466,10 +8466,10 @@
         <x:v>catalogue-63</x:v>
       </x:c>
       <x:c r="B75" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品是 ABT+2） 而且 （（出現在左半邊） 而且 （畫面沒有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品是 ABT+2） 而且 （（出現在左半邊） 而且 （背景沒有水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D75" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"all","conditions":[{"targetShape":"circle"},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"absent"}]}}]}}]}}</x:v>
@@ -8481,10 +8481,10 @@
         <x:v>catalogue-64</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 而且 （出現在左半邊）） 或 （畫面沒有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 而且 （出現在左半邊）） 或 （背景沒有水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D76" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetShape":"circle"},{"positionCondition":"left"}]}},{"distractorCondition":"absent"}]}}]}}</x:v>
@@ -8496,10 +8496,10 @@
         <x:v>catalogue-65</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C77" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 而且 （畫面沒有灰色星星）） 或 （出現在左半邊））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 而且 （背景沒有水母）） 或 （出現在左半邊））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D77" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetShape":"circle"},{"distractorCondition":"absent"}]}},{"positionCondition":"left"}]}}]}}</x:v>
@@ -8511,10 +8511,10 @@
         <x:v>catalogue-66</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>單一色環／單一商品／星星無</x:v>
+        <x:v>單一色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 而且 （畫面沒有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 而且 （背景沒有水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D78" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"absent"}]}}]}}]}}</x:v>
@@ -8526,10 +8526,10 @@
         <x:v>catalogue-67</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 或 （商品是 ABT+2）） 而且 （（出現在左半邊） 而且 （畫面有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 或 （商品是 ABT+2）） 而且 （（出現在左半邊） 而且 （背景出現水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D79" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"allowedTypes":["gold","brown"]},{"targetShape":"circle"}]}},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}</x:v>
@@ -8541,10 +8541,10 @@
         <x:v>catalogue-68</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 而且 （出現在左半邊）） 或 （（商品是 ABT+2） 或 （畫面有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 而且 （出現在左半邊）） 或 （（商品是 ABT+2） 或 （背景出現水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D80" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"allowedTypes":["gold","brown"]},{"positionCondition":"left"}]}},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"distractorCondition":"present"}]}}]}}</x:v>
@@ -8556,10 +8556,10 @@
         <x:v>catalogue-69</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C81" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 而且 （畫面有灰色星星）） 或 （（商品是 ABT+2） 或 （出現在左半邊））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 而且 （背景出現水母）） 或 （（商品是 ABT+2） 或 （出現在左半邊））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D81" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"allowedTypes":["gold","brown"]},{"distractorCondition":"present"}]}},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"positionCondition":"left"}]}}]}}</x:v>
@@ -8571,10 +8571,10 @@
         <x:v>catalogue-70</x:v>
       </x:c>
       <x:c r="B82" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（商品是 ABT+2） 或 （商品是 BBB+1））） 而且 （（出現在左半邊） 而且 （畫面有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（商品是 ABT+2） 或 （商品是 BBB+1））） 而且 （（出現在左半邊） 而且 （背景出現水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D82" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}}]}},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}</x:v>
@@ -8586,10 +8586,10 @@
         <x:v>catalogue-71</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （出現在左半邊）） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （畫面有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （出現在左半邊）） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （背景出現水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D83" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"positionCondition":"left"}]}},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"distractorCondition":"present"}]}}]}}</x:v>
@@ -8601,10 +8601,10 @@
         <x:v>catalogue-72</x:v>
       </x:c>
       <x:c r="B84" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （畫面有灰色星星）） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （出現在左半邊））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （背景出現水母）） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （出現在左半邊））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"distractorCondition":"present"}]}},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"positionCondition":"left"}]}}]}}</x:v>
@@ -8616,10 +8616,10 @@
         <x:v>catalogue-73</x:v>
       </x:c>
       <x:c r="B85" t="str">
-        <x:v>多種色環／多種商品／星星有</x:v>
+        <x:v>多種色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （（出現在左半邊） 或 （畫面有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （（出現在左半邊） 或 （背景出現水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D85" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"allowedTypes":["gold","brown"]},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"compoundCondition":{"op":"any","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}]}}</x:v>
@@ -8631,10 +8631,10 @@
         <x:v>catalogue-74</x:v>
       </x:c>
       <x:c r="B86" t="str">
-        <x:v>排除色環／單一商品／星星有</x:v>
+        <x:v>排除色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>只點符合以下條件的商品：（外圈不是金色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 或 （畫面有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈不是金色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 或 （背景出現水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D86" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"forbiddenType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"compoundCondition":{"op":"any","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}]}}</x:v>
@@ -8646,10 +8646,10 @@
         <x:v>catalogue-75</x:v>
       </x:c>
       <x:c r="B87" t="str">
-        <x:v>單一色環／排除商品／星星有</x:v>
+        <x:v>單一色環／排除商品／水母有</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品不是 ABT+2） 或 （（出現在左半邊） 或 （畫面有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（商品不是 ABT+2） 或 （（出現在左半邊） 或 （背景出現水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D87" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"forbiddenShape":"circle"},{"compoundCondition":{"op":"any","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}]}}</x:v>
@@ -8661,10 +8661,10 @@
         <x:v>catalogue-76</x:v>
       </x:c>
       <x:c r="B88" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （畫面有灰色星星）） 或 （（商品是 ABT+2） 而且 （出現在左半邊））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （背景出現水母）） 或 （（商品是 ABT+2） 而且 （出現在左半邊））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D88" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"distractorCondition":"present"}]}},{"compoundCondition":{"op":"all","conditions":[{"targetShape":"circle"},{"positionCondition":"left"}]}}]}}</x:v>
@@ -8676,10 +8676,10 @@
         <x:v>catalogue-77</x:v>
       </x:c>
       <x:c r="B89" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （出現在左半邊）） 或 （（商品是 ABT+2） 而且 （畫面有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （出現在左半邊）） 或 （（商品是 ABT+2） 而且 （背景出現水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D89" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"positionCondition":"left"}]}},{"compoundCondition":{"op":"all","conditions":[{"targetShape":"circle"},{"distractorCondition":"present"}]}}]}}</x:v>
@@ -8691,10 +8691,10 @@
         <x:v>catalogue-78</x:v>
       </x:c>
       <x:c r="B90" t="str">
-        <x:v>單一色環／單一商品／星星有</x:v>
+        <x:v>單一色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （商品是 ABT+2）） 而且 （（出現在左半邊） 或 （畫面有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （商品是 ABT+2）） 而且 （（出現在左半邊） 或 （背景出現水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D90" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"targetShape":"circle"}]}},{"compoundCondition":{"op":"any","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}</x:v>
@@ -8706,10 +8706,10 @@
         <x:v>catalogue-79</x:v>
       </x:c>
       <x:c r="B91" t="str">
-        <x:v>多種色環／單一商品／星星無</x:v>
+        <x:v>多種色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 或 （商品是 ABT+2）） 而且 （（出現在左半邊） 而且 （畫面沒有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 或 （商品是 ABT+2）） 而且 （（出現在左半邊） 而且 （背景沒有水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D91" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"allowedTypes":["gold","brown"]},{"targetShape":"circle"}]}},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"absent"}]}}]}}</x:v>
@@ -8721,10 +8721,10 @@
         <x:v>catalogue-80</x:v>
       </x:c>
       <x:c r="B92" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 或 （（商品是 ABT+2） 或 （出現在左半邊））） 而且 （畫面有灰色星星）。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 或 （（商品是 ABT+2） 或 （出現在左半邊））） 而且 （背景出現水母）。其餘不要點。</x:v>
       </x:c>
       <x:c r="D92" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"allowedTypes":["gold","brown"]},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"positionCondition":"left"}]}}]}},{"distractorCondition":"present"}]}}</x:v>
@@ -8736,10 +8736,10 @@
         <x:v>catalogue-81</x:v>
       </x:c>
       <x:c r="B93" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 或 （（商品是 ABT+2） 或 （畫面有灰色星星））） 而且 （出現在左半邊）。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 或 （（商品是 ABT+2） 或 （背景出現水母））） 而且 （出現在左半邊）。其餘不要點。</x:v>
       </x:c>
       <x:c r="D93" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"allowedTypes":["gold","brown"]},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"distractorCondition":"present"}]}}]}},{"positionCondition":"left"}]}}</x:v>
@@ -8751,10 +8751,10 @@
         <x:v>catalogue-82</x:v>
       </x:c>
       <x:c r="B94" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 而且 （（出現在左半邊） 而且 （畫面有灰色星星））） 或 （商品是 ABT+2）。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 而且 （（出現在左半邊） 而且 （背景出現水母））） 或 （商品是 ABT+2）。其餘不要點。</x:v>
       </x:c>
       <x:c r="D94" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"allowedTypes":["gold","brown"]},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}},{"targetShape":"circle"}]}}</x:v>
@@ -8766,10 +8766,10 @@
         <x:v>catalogue-83</x:v>
       </x:c>
       <x:c r="B95" t="str">
-        <x:v>多種色環／單一商品／星星無</x:v>
+        <x:v>多種色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 而且 （出現在左半邊）） 或 （（商品是 ABT+2） 或 （畫面沒有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 而且 （出現在左半邊）） 或 （（商品是 ABT+2） 或 （背景沒有水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D95" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"allowedTypes":["gold","brown"]},{"positionCondition":"left"}]}},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"distractorCondition":"absent"}]}}]}}</x:v>
@@ -8781,10 +8781,10 @@
         <x:v>catalogue-84</x:v>
       </x:c>
       <x:c r="B96" t="str">
-        <x:v>多種色環／單一商品／星星無</x:v>
+        <x:v>多種色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 而且 （畫面沒有灰色星星）） 或 （（商品是 ABT+2） 或 （出現在左半邊））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色、棕色其中一色） 而且 （背景沒有水母）） 或 （（商品是 ABT+2） 或 （出現在左半邊））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D96" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"allowedTypes":["gold","brown"]},{"distractorCondition":"absent"}]}},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"positionCondition":"left"}]}}]}}</x:v>
@@ -8796,10 +8796,10 @@
         <x:v>catalogue-85</x:v>
       </x:c>
       <x:c r="B97" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（商品是 ABT+2） 而且 （（出現在左半邊） 而且 （畫面有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（商品是 ABT+2） 而且 （（出現在左半邊） 而且 （背景出現水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D97" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"allowedTypes":["gold","brown"]},{"compoundCondition":{"op":"all","conditions":[{"targetShape":"circle"},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}]}}</x:v>
@@ -8811,10 +8811,10 @@
         <x:v>catalogue-86</x:v>
       </x:c>
       <x:c r="B98" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（（商品是 ABT+2） 而且 （出現在左半邊）） 或 （畫面有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（（商品是 ABT+2） 而且 （出現在左半邊）） 或 （背景出現水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D98" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"allowedTypes":["gold","brown"]},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetShape":"circle"},{"positionCondition":"left"}]}},{"distractorCondition":"present"}]}}]}}</x:v>
@@ -8826,10 +8826,10 @@
         <x:v>catalogue-87</x:v>
       </x:c>
       <x:c r="B99" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（（商品是 ABT+2） 而且 （畫面有灰色星星）） 或 （出現在左半邊））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（（商品是 ABT+2） 而且 （背景出現水母）） 或 （出現在左半邊））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D99" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"allowedTypes":["gold","brown"]},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetShape":"circle"},{"distractorCondition":"present"}]}},{"positionCondition":"left"}]}}]}}</x:v>
@@ -8841,10 +8841,10 @@
         <x:v>catalogue-88</x:v>
       </x:c>
       <x:c r="B100" t="str">
-        <x:v>多種色環／單一商品／星星有</x:v>
+        <x:v>多種色環／單一商品／水母有</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 而且 （畫面有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 而且 （背景出現水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D100" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"allowedTypes":["gold","brown"]},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}]}}</x:v>
@@ -8856,10 +8856,10 @@
         <x:v>catalogue-89</x:v>
       </x:c>
       <x:c r="B101" t="str">
-        <x:v>單一色環／多種商品／星星無</x:v>
+        <x:v>單一色環／多種商品／水母無</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（商品是 ABT+2） 或 （商品是 BBB+1））） 而且 （（出現在左半邊） 而且 （畫面沒有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（商品是 ABT+2） 或 （商品是 BBB+1））） 而且 （（出現在左半邊） 而且 （背景沒有水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D101" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}}]}},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"absent"}]}}]}}</x:v>
@@ -8871,10 +8871,10 @@
         <x:v>catalogue-90</x:v>
       </x:c>
       <x:c r="B102" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （出現在左半邊））） 而且 （畫面有灰色星星）。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （出現在左半邊））） 而且 （背景出現水母）。其餘不要點。</x:v>
       </x:c>
       <x:c r="D102" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"positionCondition":"left"}]}}]}},{"distractorCondition":"present"}]}}</x:v>
@@ -8886,10 +8886,10 @@
         <x:v>catalogue-91</x:v>
       </x:c>
       <x:c r="B103" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （畫面有灰色星星））） 而且 （出現在左半邊）。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （背景出現水母））） 而且 （出現在左半邊）。其餘不要點。</x:v>
       </x:c>
       <x:c r="D103" t="str">
         <x:v>{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"distractorCondition":"present"}]}}]}},{"positionCondition":"left"}]}}</x:v>
@@ -8901,10 +8901,10 @@
         <x:v>catalogue-92</x:v>
       </x:c>
       <x:c r="B104" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （（出現在左半邊） 而且 （畫面有灰色星星））） 或 （（商品是 ABT+2） 或 （商品是 BBB+1））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （（出現在左半邊） 而且 （背景出現水母））） 或 （（商品是 ABT+2） 或 （商品是 BBB+1））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D104" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}}]}}</x:v>
@@ -8916,10 +8916,10 @@
         <x:v>catalogue-93</x:v>
       </x:c>
       <x:c r="B105" t="str">
-        <x:v>單一色環／多種商品／星星無</x:v>
+        <x:v>單一色環／多種商品／水母無</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （出現在左半邊）） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （畫面沒有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （出現在左半邊）） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （背景沒有水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D105" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"positionCondition":"left"}]}},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"distractorCondition":"absent"}]}}]}}</x:v>
@@ -8931,10 +8931,10 @@
         <x:v>catalogue-94</x:v>
       </x:c>
       <x:c r="B106" t="str">
-        <x:v>單一色環／多種商品／星星無</x:v>
+        <x:v>單一色環／多種商品／水母無</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （畫面沒有灰色星星）） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （出現在左半邊））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（（外圈是金色） 而且 （背景沒有水母）） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （出現在左半邊））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D106" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"targetType":"gold"},{"distractorCondition":"absent"}]}},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"positionCondition":"left"}]}}]}}</x:v>
@@ -8946,10 +8946,10 @@
         <x:v>catalogue-95</x:v>
       </x:c>
       <x:c r="B107" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 而且 （（出現在左半邊） 而且 （畫面有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 而且 （（出現在左半邊） 而且 （背景出現水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D107" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}]}}</x:v>
@@ -8961,10 +8961,10 @@
         <x:v>catalogue-96</x:v>
       </x:c>
       <x:c r="B108" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（（商品是 ABT+2） 或 （商品是 BBB+1）） 而且 （出現在左半邊）） 或 （畫面有灰色星星））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（（商品是 ABT+2） 或 （商品是 BBB+1）） 而且 （出現在左半邊）） 或 （背景出現水母））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D108" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"positionCondition":"left"}]}},{"distractorCondition":"present"}]}}]}}</x:v>
@@ -8976,10 +8976,10 @@
         <x:v>catalogue-97</x:v>
       </x:c>
       <x:c r="B109" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（（商品是 ABT+2） 或 （商品是 BBB+1）） 而且 （畫面有灰色星星）） 或 （出現在左半邊））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（（商品是 ABT+2） 或 （商品是 BBB+1）） 而且 （背景出現水母）） 或 （出現在左半邊））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D109" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"all","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"distractorCondition":"present"}]}},{"positionCondition":"left"}]}}]}}</x:v>
@@ -8991,10 +8991,10 @@
         <x:v>catalogue-98</x:v>
       </x:c>
       <x:c r="B110" t="str">
-        <x:v>單一色環／多種商品／星星有</x:v>
+        <x:v>單一色環／多種商品／水母有</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （（出現在左半邊） 而且 （畫面有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （（出現在左半邊） 而且 （背景出現水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D110" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"compoundCondition":{"op":"all","conditions":[{"positionCondition":"left"},{"distractorCondition":"present"}]}}]}}]}}</x:v>
@@ -9006,10 +9006,10 @@
         <x:v>catalogue-99</x:v>
       </x:c>
       <x:c r="B111" t="str">
-        <x:v>多種色環／多種商品／星星無</x:v>
+        <x:v>多種色環／多種商品／水母無</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （（出現在左半邊） 或 （畫面沒有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈是金色、棕色其中一色） 或 （（（商品是 ABT+2） 或 （商品是 BBB+1）） 或 （（出現在左半邊） 或 （背景沒有水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D111" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"allowedTypes":["gold","brown"]},{"compoundCondition":{"op":"any","conditions":[{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}},{"compoundCondition":{"op":"any","conditions":[{"positionCondition":"left"},{"distractorCondition":"absent"}]}}]}}]}}</x:v>
@@ -9021,10 +9021,10 @@
         <x:v>catalogue-100</x:v>
       </x:c>
       <x:c r="B112" t="str">
-        <x:v>排除色環／單一商品／星星無</x:v>
+        <x:v>排除色環／單一商品／水母無</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>只點符合以下條件的商品：（外圈不是金色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 或 （畫面沒有灰色星星）））。其餘不要點。</x:v>
+        <x:v>只點符合以下條件的商品：（外圈不是金色） 或 （（商品是 ABT+2） 或 （（出現在左半邊） 或 （背景沒有水母）））。其餘不要點。</x:v>
       </x:c>
       <x:c r="D112" t="str">
         <x:v>{"compoundCondition":{"op":"any","conditions":[{"forbiddenType":"gold"},{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"compoundCondition":{"op":"any","conditions":[{"positionCondition":"left"},{"distractorCondition":"absent"}]}}]}}]}}</x:v>
@@ -9997,6 +9997,9 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:cols>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
@@ -10108,13 +10111,13 @@
         <x:v>distractor</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>noise.svg</x:v>
+        <x:v>jellyfish.webp</x:v>
       </x:c>
       <x:c r="D7" t="b">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>灰色星星</x:v>
+        <x:v>背景水母</x:v>
       </x:c>
     </x:row>
     <x:row r="8">

</xml_diff>

<commit_message>
Add nine single-rule beginner tutorials with separate progress
</commit_message>
<xml_diff>
--- a/games/reaction-speed-test/config/game_config.xlsx
+++ b/games/reaction-speed-test/config/game_config.xlsx
@@ -2,15 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameSettings" sheetId="1" r:id="R72f4aad1411042e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="2" r:id="R2514fc28e82a44ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R47b0226a1c304036"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stimuli" sheetId="4" r:id="R3eed6c1e6ac34829"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InfiniteMode" sheetId="5" r:id="R9b5359be32b34b39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rdda6b7ef4a4e47a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="7" r:id="Rbad9383c31034f9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="8" r:id="R0eefa96c359f4410"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Text" sheetId="9" r:id="Rccc079b5353b42c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameSettings" sheetId="1" r:id="R64b17cae067f423e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levels" sheetId="2" r:id="Rca817989747e4c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="3" r:id="R41815f9856164546"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stimuli" sheetId="4" r:id="R2a3b32e3c8804ee1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InfiniteMode" sheetId="5" r:id="Rdaff70aef79545e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="6" r:id="Rfbb2623a64364a8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Animations" sheetId="7" r:id="R0f856f7db339437b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audio" sheetId="8" r:id="Rc10032bd992b4ea0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Text" sheetId="9" r:id="R6202214ce13a47d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tutorials" sheetId="10" r:id="R5c80af1923ab476b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43,22 +44,39 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <x:numFmt numFmtId="200" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="1">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="12"/>
       <x:color theme="1"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="Microsoft JhengHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFF5F0E6"/>
+      <x:name val="Microsoft JhengHei"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="2">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF46634F"/>
+      </x:patternFill>
     </x:fill>
   </x:fills>
   <x:borders count="1">
@@ -67,7 +85,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="2">
+  <x:cellXfs count="8">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <x:extLst>
@@ -76,6 +94,20 @@
         </x:ext>
       </x:extLst>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -448,6 +480,626 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="82" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="22" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="22" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="22" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="6" t="str">
+        <x:v>levelId</x:v>
+      </x:c>
+      <x:c r="B1" s="6" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="C1" s="6" t="str">
+        <x:v>ruleId</x:v>
+      </x:c>
+      <x:c r="D1" s="6" t="str">
+        <x:v>condition</x:v>
+      </x:c>
+      <x:c r="E1" s="6" t="str">
+        <x:v>stimulusCount</x:v>
+      </x:c>
+      <x:c r="F1" s="6" t="str">
+        <x:v>timeLimit</x:v>
+      </x:c>
+      <x:c r="G1" s="6" t="str">
+        <x:v>minInterval</x:v>
+      </x:c>
+      <x:c r="H1" s="6" t="str">
+        <x:v>maxInterval</x:v>
+      </x:c>
+      <x:c r="I1" s="6" t="str">
+        <x:v>stimulusDuration</x:v>
+      </x:c>
+      <x:c r="J1" s="6" t="str">
+        <x:v>requiredAccuracy</x:v>
+      </x:c>
+      <x:c r="K1" s="6" t="str">
+        <x:v>targetRatio</x:v>
+      </x:c>
+      <x:c r="L1" s="6" t="str">
+        <x:v>distractorRatio</x:v>
+      </x:c>
+      <x:c r="M1" s="6" t="str">
+        <x:v>randomPosition</x:v>
+      </x:c>
+      <x:c r="N1" s="6" t="str">
+        <x:v>countdownEnabled</x:v>
+      </x:c>
+      <x:c r="O1" s="6" t="str">
+        <x:v>enabled</x:v>
+      </x:c>
+      <x:c r="P1" s="6" t="str">
+        <x:v>randomizeTargets</x:v>
+      </x:c>
+      <x:c r="Q1" s="6" t="str">
+        <x:v>starAccuracy</x:v>
+      </x:c>
+      <x:c r="R1" s="6" t="str">
+        <x:v>starAverageMs</x:v>
+      </x:c>
+      <x:c r="S1" s="6" t="str">
+        <x:v>ruleRevision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="52" customHeight="1">
+      <x:c r="A2" s="2" t="str">
+        <x:v>tutorial-1</x:v>
+      </x:c>
+      <x:c r="B2" s="2" t="str">
+        <x:v>指定一種色環</x:v>
+      </x:c>
+      <x:c r="C2" s="2" t="str">
+        <x:v>tutorial-rule-1</x:v>
+      </x:c>
+      <x:c r="D2" s="4" t="str">
+        <x:v>{"targetType":"gold"}</x:v>
+      </x:c>
+      <x:c r="E2" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F2" s="2" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G2" s="2" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="H2" s="2" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="I2" s="2" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J2" s="2" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="K2" s="2" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="L2" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M2" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N2" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O2" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P2" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q2" s="7" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="R2" s="2" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="S2" s="2" t="str">
+        <x:v>tutorial-v1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="52" customHeight="1">
+      <x:c r="A3" s="2" t="str">
+        <x:v>tutorial-2</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="str">
+        <x:v>指定多種色環</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="str">
+        <x:v>tutorial-rule-2</x:v>
+      </x:c>
+      <x:c r="D3" s="4" t="str">
+        <x:v>{"allowedTypes":["gold","blue"]}</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F3" s="2" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G3" s="2" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="H3" s="2" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="I3" s="2" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J3" s="2" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="K3" s="2" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="L3" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M3" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N3" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O3" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P3" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q3" s="7" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="R3" s="2" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="S3" s="2" t="str">
+        <x:v>tutorial-v1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="52" customHeight="1">
+      <x:c r="A4" s="2" t="str">
+        <x:v>tutorial-3</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="str">
+        <x:v>排除一種色環</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="str">
+        <x:v>tutorial-rule-3</x:v>
+      </x:c>
+      <x:c r="D4" s="4" t="str">
+        <x:v>{"forbiddenType":"red"}</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G4" s="2" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="H4" s="2" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="I4" s="2" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J4" s="2" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="K4" s="2" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="L4" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M4" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N4" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O4" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P4" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q4" s="7" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="R4" s="2" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="S4" s="2" t="str">
+        <x:v>tutorial-v1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="52" customHeight="1">
+      <x:c r="A5" s="2" t="str">
+        <x:v>tutorial-4</x:v>
+      </x:c>
+      <x:c r="B5" s="2" t="str">
+        <x:v>指定一種商品</x:v>
+      </x:c>
+      <x:c r="C5" s="2" t="str">
+        <x:v>tutorial-rule-4</x:v>
+      </x:c>
+      <x:c r="D5" s="4" t="str">
+        <x:v>{"targetShape":"circle"}</x:v>
+      </x:c>
+      <x:c r="E5" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F5" s="2" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G5" s="2" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="H5" s="2" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="I5" s="2" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J5" s="2" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="K5" s="2" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="L5" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M5" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N5" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O5" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P5" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q5" s="7" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="R5" s="2" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="S5" s="2" t="str">
+        <x:v>tutorial-v1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="52" customHeight="1">
+      <x:c r="A6" s="2" t="str">
+        <x:v>tutorial-5</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="str">
+        <x:v>指定多種商品</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="str">
+        <x:v>tutorial-rule-5</x:v>
+      </x:c>
+      <x:c r="D6" s="4" t="str">
+        <x:v>{"compoundCondition":{"op":"any","conditions":[{"targetShape":"circle"},{"targetShape":"square"}]}}</x:v>
+      </x:c>
+      <x:c r="E6" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F6" s="2" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G6" s="2" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="H6" s="2" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="I6" s="2" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J6" s="2" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="K6" s="2" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="L6" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M6" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N6" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O6" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P6" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q6" s="7" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="R6" s="2" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="S6" s="2" t="str">
+        <x:v>tutorial-v1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="52" customHeight="1">
+      <x:c r="A7" s="2" t="str">
+        <x:v>tutorial-6</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="str">
+        <x:v>排除一種商品</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="str">
+        <x:v>tutorial-rule-6</x:v>
+      </x:c>
+      <x:c r="D7" s="4" t="str">
+        <x:v>{"forbiddenShape":"triangle"}</x:v>
+      </x:c>
+      <x:c r="E7" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F7" s="2" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G7" s="2" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="H7" s="2" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="I7" s="2" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J7" s="2" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="K7" s="2" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="L7" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M7" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N7" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O7" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P7" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q7" s="7" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="R7" s="2" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="S7" s="2" t="str">
+        <x:v>tutorial-v1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="52" customHeight="1">
+      <x:c r="A8" s="2" t="str">
+        <x:v>tutorial-7</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="str">
+        <x:v>只點指定側</x:v>
+      </x:c>
+      <x:c r="C8" s="2" t="str">
+        <x:v>tutorial-rule-7</x:v>
+      </x:c>
+      <x:c r="D8" s="4" t="str">
+        <x:v>{"positionCondition":"left"}</x:v>
+      </x:c>
+      <x:c r="E8" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F8" s="2" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G8" s="2" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="H8" s="2" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="I8" s="2" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J8" s="2" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="K8" s="2" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="L8" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M8" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N8" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O8" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P8" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q8" s="7" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="R8" s="2" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="S8" s="2" t="str">
+        <x:v>tutorial-v1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="52" customHeight="1">
+      <x:c r="A9" s="2" t="str">
+        <x:v>tutorial-8</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="str">
+        <x:v>背景有水母</x:v>
+      </x:c>
+      <x:c r="C9" s="2" t="str">
+        <x:v>tutorial-rule-8</x:v>
+      </x:c>
+      <x:c r="D9" s="4" t="str">
+        <x:v>{"distractorCondition":"present"}</x:v>
+      </x:c>
+      <x:c r="E9" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F9" s="2" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G9" s="2" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="H9" s="2" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="I9" s="2" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J9" s="2" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="K9" s="2" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="L9" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="M9" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N9" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O9" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P9" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q9" s="7" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="R9" s="2" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="S9" s="2" t="str">
+        <x:v>tutorial-v1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="52" customHeight="1">
+      <x:c r="A10" s="2" t="str">
+        <x:v>tutorial-9</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="str">
+        <x:v>背景沒有水母</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:v>tutorial-rule-9</x:v>
+      </x:c>
+      <x:c r="D10" s="4" t="str">
+        <x:v>{"distractorCondition":"absent"}</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F10" s="2" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G10" s="2" t="n">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="H10" s="2" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="I10" s="2" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="J10" s="2" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="K10" s="2" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="L10" s="2" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="M10" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N10" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O10" s="3" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P10" s="3" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q10" s="7" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="R10" s="2" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="S10" s="2" t="str">
+        <x:v>tutorial-v1</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:cols>

</xml_diff>